<commit_message>
Verification experiments save point.
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -60,7 +60,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -149,6 +149,11 @@
           <t>years to transition ats</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>profit margin</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -167,40 +172,43 @@
         <v>0.7</v>
       </c>
       <c r="F2" t="n">
-        <v>7.0</v>
+        <v>9.59217253160857</v>
       </c>
       <c r="G2" t="n">
-        <v>3.6687854661123813</v>
+        <v>8.393616962771578</v>
       </c>
       <c r="H2" t="n">
-        <v>3.036354611073011</v>
+        <v>5.995702918702903</v>
       </c>
       <c r="I2" t="n">
-        <v>50.0</v>
+        <v>159.17100275103942</v>
       </c>
       <c r="J2" t="n">
-        <v>50.0</v>
+        <v>144.42540564720525</v>
       </c>
       <c r="K2" t="n">
-        <v>50.0</v>
+        <v>108.44527521712024</v>
       </c>
       <c r="L2" t="n">
         <v>0.0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.074378311174592</v>
+        <v>0.09400847705046052</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7836673784769767</v>
+        <v>0.7837580175461181</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7107624561038625</v>
+        <v>0.7111506974068387</v>
       </c>
       <c r="P2" t="n">
         <v>0.5339845351691</v>
       </c>
       <c r="Q2" t="n">
         <v>25.0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">
@@ -220,40 +228,43 @@
         <v>0.7</v>
       </c>
       <c r="F3" t="n">
-        <v>9.485901677703112</v>
+        <v>10.246015625138003</v>
       </c>
       <c r="G3" t="n">
-        <v>8.897348088767941</v>
+        <v>8.654383431501124</v>
       </c>
       <c r="H3" t="n">
-        <v>7.0</v>
+        <v>5.995702918702903</v>
       </c>
       <c r="I3" t="n">
-        <v>150.0</v>
+        <v>174.34313093409196</v>
       </c>
       <c r="J3" t="n">
-        <v>150.0</v>
+        <v>146.1507987542513</v>
       </c>
       <c r="K3" t="n">
-        <v>150.0</v>
+        <v>108.44527521712024</v>
       </c>
       <c r="L3" t="n">
         <v>0.0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.39062288206894125</v>
+        <v>0.38049498236678936</v>
       </c>
       <c r="N3" t="n">
-        <v>0.8608968250980082</v>
+        <v>0.8584655767194689</v>
       </c>
       <c r="O3" t="n">
-        <v>0.720173909128709</v>
+        <v>0.7196465330659335</v>
       </c>
       <c r="P3" t="n">
         <v>0.5339845351691</v>
       </c>
       <c r="Q3" t="n">
         <v>25.0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="4">
@@ -273,40 +284,43 @@
         <v>0.7</v>
       </c>
       <c r="F4" t="n">
-        <v>7.0</v>
+        <v>9.908336098022382</v>
       </c>
       <c r="G4" t="n">
-        <v>6.310206048183373</v>
+        <v>8.531879085280357</v>
       </c>
       <c r="H4" t="n">
-        <v>5.592853230563756</v>
+        <v>5.995702918702903</v>
       </c>
       <c r="I4" t="n">
-        <v>100.0</v>
+        <v>165.42721203353108</v>
       </c>
       <c r="J4" t="n">
-        <v>100.0</v>
+        <v>145.18328430147182</v>
       </c>
       <c r="K4" t="n">
-        <v>100.0</v>
+        <v>108.44527521712024</v>
       </c>
       <c r="L4" t="n">
         <v>0.0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.20570672405411677</v>
+        <v>0.1976116120986026</v>
       </c>
       <c r="N4" t="n">
-        <v>0.8165068604892819</v>
+        <v>0.814563592053107</v>
       </c>
       <c r="O4" t="n">
-        <v>0.7153885453847253</v>
+        <v>0.714882491900447</v>
       </c>
       <c r="P4" t="n">
         <v>0.5339845351691</v>
       </c>
       <c r="Q4" t="n">
         <v>25.0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sensitivity test for starting capacity.
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -60,7 +60,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -181,49 +181,49 @@
         <v>0.1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E2" t="n">
         <v>0.7</v>
       </c>
       <c r="F2" t="n">
-        <v>36.28940687876643</v>
+        <v>28.41097645332293</v>
       </c>
       <c r="G2" t="n">
-        <v>19.716959407525085</v>
+        <v>16.50237684348026</v>
       </c>
       <c r="H2" t="n">
-        <v>12.541144704611776</v>
+        <v>10.545823234677838</v>
       </c>
       <c r="I2" t="n">
-        <v>234.28749518938986</v>
+        <v>195.2795744295943</v>
       </c>
       <c r="J2" t="n">
-        <v>189.39065061880427</v>
+        <v>147.5371247524124</v>
       </c>
       <c r="K2" t="n">
-        <v>111.67769253169617</v>
+        <v>105.94417321878504</v>
       </c>
       <c r="L2" t="n">
         <v>0.0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9978058397019188</v>
+        <v>0.9486999753389981</v>
       </c>
       <c r="N2" t="n">
-        <v>1.1536316263125557</v>
+        <v>0.9615566244913223</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9325595636469917</v>
+        <v>0.7264728022808785</v>
       </c>
       <c r="P2" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5216691089292975</v>
       </c>
       <c r="Q2" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R2" t="n">
-        <v>4950000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S2" t="n">
         <v>0.08</v>
@@ -246,49 +246,49 @@
         <v>0.1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E3" t="n">
         <v>0.7</v>
       </c>
       <c r="F3" t="n">
-        <v>36.3020449623616</v>
+        <v>29.780783977693822</v>
       </c>
       <c r="G3" t="n">
-        <v>19.71718696925032</v>
+        <v>15.58365163678584</v>
       </c>
       <c r="H3" t="n">
-        <v>12.54087422740917</v>
+        <v>10.496061526398798</v>
       </c>
       <c r="I3" t="n">
-        <v>234.28892298163802</v>
+        <v>195.28693645821852</v>
       </c>
       <c r="J3" t="n">
-        <v>189.39404328589242</v>
+        <v>148.27430970996303</v>
       </c>
       <c r="K3" t="n">
-        <v>111.67769253169617</v>
+        <v>105.96533559259294</v>
       </c>
       <c r="L3" t="n">
         <v>0.0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9978350318503323</v>
+        <v>0.9488662965098728</v>
       </c>
       <c r="N3" t="n">
-        <v>1.1536386567615855</v>
+        <v>0.9615928751202679</v>
       </c>
       <c r="O3" t="n">
-        <v>0.9325762691397338</v>
+        <v>0.730102701011858</v>
       </c>
       <c r="P3" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5217733124579276</v>
       </c>
       <c r="Q3" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R3" t="n">
-        <v>5850000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S3" t="n">
         <v>0.08</v>
@@ -311,49 +311,49 @@
         <v>0.1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E4" t="n">
         <v>0.7</v>
       </c>
       <c r="F4" t="n">
-        <v>36.31465847197772</v>
+        <v>29.969710495299793</v>
       </c>
       <c r="G4" t="n">
-        <v>19.717425829949526</v>
+        <v>16.964644979867217</v>
       </c>
       <c r="H4" t="n">
-        <v>12.540601633338504</v>
+        <v>10.60809208186763</v>
       </c>
       <c r="I4" t="n">
-        <v>234.29036139475036</v>
+        <v>195.2790628606574</v>
       </c>
       <c r="J4" t="n">
-        <v>189.39744306854502</v>
+        <v>146.95659545461845</v>
       </c>
       <c r="K4" t="n">
-        <v>111.67769253169617</v>
+        <v>105.81719897593761</v>
       </c>
       <c r="L4" t="n">
         <v>0.0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9978644411492771</v>
+        <v>0.9486884180972501</v>
       </c>
       <c r="N4" t="n">
-        <v>1.1536457395077508</v>
+        <v>0.9615541055258771</v>
       </c>
       <c r="O4" t="n">
-        <v>0.9325930096695163</v>
+        <v>0.7236142760185416</v>
       </c>
       <c r="P4" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5210438877575169</v>
       </c>
       <c r="Q4" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R4" t="n">
-        <v>6750000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S4" t="n">
         <v>0.08</v>
@@ -376,49 +376,49 @@
         <v>0.1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E5" t="n">
         <v>0.7</v>
       </c>
       <c r="F5" t="n">
-        <v>36.225843068145316</v>
+        <v>30.21357635776602</v>
       </c>
       <c r="G5" t="n">
-        <v>19.715383031408205</v>
+        <v>16.694586352223947</v>
       </c>
       <c r="H5" t="n">
-        <v>12.542484764540083</v>
+        <v>10.553937002892145</v>
       </c>
       <c r="I5" t="n">
-        <v>234.28051554111343</v>
+        <v>195.28145804737852</v>
       </c>
       <c r="J5" t="n">
-        <v>189.37547610345476</v>
+        <v>147.3502025453923</v>
       </c>
       <c r="K5" t="n">
-        <v>111.67769253169617</v>
+        <v>105.90184847116923</v>
       </c>
       <c r="L5" t="n">
         <v>0.0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.9976631362178284</v>
+        <v>0.9487425295766067</v>
       </c>
       <c r="N5" t="n">
-        <v>1.1535972585244425</v>
+        <v>0.9615658994252918</v>
       </c>
       <c r="O5" t="n">
-        <v>0.9324848443334113</v>
+        <v>0.7255523973335115</v>
       </c>
       <c r="P5" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5214607018720373</v>
       </c>
       <c r="Q5" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R5" t="n">
-        <v>450000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S5" t="n">
         <v>0.08</v>
@@ -441,49 +441,49 @@
         <v>0.1</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E6" t="n">
         <v>0.7</v>
       </c>
       <c r="F6" t="n">
-        <v>36.276744085542035</v>
+        <v>29.473923819084238</v>
       </c>
       <c r="G6" t="n">
-        <v>19.716743268394055</v>
+        <v>16.63690746801699</v>
       </c>
       <c r="H6" t="n">
-        <v>12.541413064590323</v>
+        <v>10.552466485108072</v>
       </c>
       <c r="I6" t="n">
-        <v>234.28607801800604</v>
+        <v>195.27244450605397</v>
       </c>
       <c r="J6" t="n">
-        <v>189.38726506728088</v>
+        <v>147.44248471645096</v>
       </c>
       <c r="K6" t="n">
-        <v>111.67769253169617</v>
+        <v>105.92301084497716</v>
       </c>
       <c r="L6" t="n">
         <v>0.0</v>
       </c>
       <c r="M6" t="n">
-        <v>0.9977768647040371</v>
+        <v>0.9485388978300666</v>
       </c>
       <c r="N6" t="n">
-        <v>1.1536246481606618</v>
+        <v>0.9615215167478097</v>
       </c>
       <c r="O6" t="n">
-        <v>0.9325428931912905</v>
+        <v>0.7260067947438049</v>
       </c>
       <c r="P6" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5215649054006675</v>
       </c>
       <c r="Q6" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R6" t="n">
-        <v>4050000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S6" t="n">
         <v>0.08</v>
@@ -506,49 +506,49 @@
         <v>0.1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E7" t="n">
         <v>0.7</v>
       </c>
       <c r="F7" t="n">
-        <v>36.26405644603796</v>
+        <v>30.186549959802534</v>
       </c>
       <c r="G7" t="n">
-        <v>19.716538677065525</v>
+        <v>16.72682945211705</v>
       </c>
       <c r="H7" t="n">
-        <v>12.541679306991535</v>
+        <v>10.568203666168559</v>
       </c>
       <c r="I7" t="n">
-        <v>234.28467146748648</v>
+        <v>195.27467677153132</v>
       </c>
       <c r="J7" t="n">
-        <v>189.38388663132193</v>
+        <v>147.25758584736147</v>
       </c>
       <c r="K7" t="n">
-        <v>111.67769253169617</v>
+        <v>105.88068609736135</v>
       </c>
       <c r="L7" t="n">
         <v>0.0</v>
       </c>
       <c r="M7" t="n">
-        <v>0.9977481068566875</v>
+        <v>0.9485893286320701</v>
       </c>
       <c r="N7" t="n">
-        <v>1.1536177223059034</v>
+        <v>0.9615325084230202</v>
       </c>
       <c r="O7" t="n">
-        <v>0.9325262577726294</v>
+        <v>0.7250963527124079</v>
       </c>
       <c r="P7" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5213564983434072</v>
       </c>
       <c r="Q7" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R7" t="n">
-        <v>3150000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S7" t="n">
         <v>0.08</v>
@@ -571,49 +571,49 @@
         <v>0.1</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E8" t="n">
         <v>0.7</v>
       </c>
       <c r="F8" t="n">
-        <v>36.25134382259434</v>
+        <v>30.15983371065964</v>
       </c>
       <c r="G8" t="n">
-        <v>19.715733421478888</v>
+        <v>16.796471807428038</v>
       </c>
       <c r="H8" t="n">
-        <v>12.541962868810614</v>
+        <v>10.597017881571995</v>
       </c>
       <c r="I8" t="n">
-        <v>234.28327553783114</v>
+        <v>195.28403909715703</v>
       </c>
       <c r="J8" t="n">
-        <v>189.38219739754905</v>
+        <v>147.16222209971895</v>
       </c>
       <c r="K8" t="n">
-        <v>111.67769253169617</v>
+        <v>105.85952372355341</v>
       </c>
       <c r="L8" t="n">
         <v>0.0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.9977195661598692</v>
+        <v>0.9488008400292219</v>
       </c>
       <c r="N8" t="n">
-        <v>1.1536108487482806</v>
+        <v>0.9615786085144012</v>
       </c>
       <c r="O8" t="n">
-        <v>0.9325179399855309</v>
+        <v>0.7246267816190165</v>
       </c>
       <c r="P8" t="n">
-        <v>0.549900958026072</v>
+        <v>0.521252294814777</v>
       </c>
       <c r="Q8" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R8" t="n">
-        <v>2250000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S8" t="n">
         <v>0.08</v>
@@ -636,49 +636,49 @@
         <v>0.1</v>
       </c>
       <c r="D9" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E9" t="n">
         <v>0.7</v>
       </c>
       <c r="F9" t="n">
-        <v>36.23860607653245</v>
+        <v>28.56673852253458</v>
       </c>
       <c r="G9" t="n">
-        <v>19.715552259654807</v>
+        <v>15.478079803252363</v>
       </c>
       <c r="H9" t="n">
-        <v>12.54222487598942</v>
+        <v>10.496878473593608</v>
       </c>
       <c r="I9" t="n">
-        <v>234.2818902290402</v>
+        <v>195.28585880641012</v>
       </c>
       <c r="J9" t="n">
-        <v>189.37883319271955</v>
+        <v>148.32820990917693</v>
       </c>
       <c r="K9" t="n">
-        <v>111.67769253169617</v>
+        <v>106.00766034020876</v>
       </c>
       <c r="L9" t="n">
         <v>0.0</v>
       </c>
       <c r="M9" t="n">
-        <v>0.9976912426135828</v>
+        <v>0.9488419504607455</v>
       </c>
       <c r="N9" t="n">
-        <v>1.153604027487794</v>
+        <v>0.9615875687627634</v>
       </c>
       <c r="O9" t="n">
-        <v>0.9325013746409511</v>
+        <v>0.7303681055927874</v>
       </c>
       <c r="P9" t="n">
-        <v>0.549900958026072</v>
+        <v>0.521981719515188</v>
       </c>
       <c r="Q9" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R9" t="n">
-        <v>1350000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S9" t="n">
         <v>0.08</v>
@@ -701,49 +701,49 @@
         <v>0.1</v>
       </c>
       <c r="D10" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E10" t="n">
         <v>0.7</v>
       </c>
       <c r="F10" t="n">
-        <v>36.339812306927044</v>
+        <v>29.867460380569</v>
       </c>
       <c r="G10" t="n">
-        <v>19.71932361272845</v>
+        <v>16.880881194352394</v>
       </c>
       <c r="H10" t="n">
-        <v>12.543240682792895</v>
+        <v>10.605308784976822</v>
       </c>
       <c r="I10" t="n">
-        <v>234.27730091170406</v>
+        <v>195.27341471283276</v>
       </c>
       <c r="J10" t="n">
-        <v>189.39894092325687</v>
+        <v>147.04566799527734</v>
       </c>
       <c r="K10" t="n">
-        <v>111.67769253169617</v>
+        <v>105.83836134974551</v>
       </c>
       <c r="L10" t="n">
         <v>0.0</v>
       </c>
       <c r="M10" t="n">
-        <v>0.997597411012404</v>
+        <v>0.9485608165070605</v>
       </c>
       <c r="N10" t="n">
-        <v>1.1535814296892308</v>
+        <v>0.9615262940459884</v>
       </c>
       <c r="O10" t="n">
-        <v>0.9326003851061165</v>
+        <v>0.7240528692087459</v>
       </c>
       <c r="P10" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5211480912861469</v>
       </c>
       <c r="Q10" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R10" t="n">
-        <v>8550000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S10" t="n">
         <v>0.08</v>
@@ -766,49 +766,49 @@
         <v>0.1</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E11" t="n">
         <v>0.7</v>
       </c>
       <c r="F11" t="n">
-        <v>36.35235289864115</v>
+        <v>28.45887060621136</v>
       </c>
       <c r="G11" t="n">
-        <v>19.72024710465626</v>
+        <v>15.351650585600195</v>
       </c>
       <c r="H11" t="n">
-        <v>12.543011440699166</v>
+        <v>10.47846629169804</v>
       </c>
       <c r="I11" t="n">
-        <v>234.27877118740926</v>
+        <v>195.28487326228222</v>
       </c>
       <c r="J11" t="n">
-        <v>189.40057699696908</v>
+        <v>148.3824076567449</v>
       </c>
       <c r="K11" t="n">
-        <v>111.67769253169617</v>
+        <v>106.04998508782455</v>
       </c>
       <c r="L11" t="n">
         <v>0.0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.9976274717629443</v>
+        <v>0.9488196852860675</v>
       </c>
       <c r="N11" t="n">
-        <v>1.1535886693268032</v>
+        <v>0.9615827159434777</v>
       </c>
       <c r="O11" t="n">
-        <v>0.9326084411330765</v>
+        <v>0.7306349753018117</v>
       </c>
       <c r="P11" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5221901265724481</v>
       </c>
       <c r="Q11" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R11" t="n">
-        <v>9450000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S11" t="n">
         <v>0.08</v>
@@ -831,49 +831,49 @@
         <v>0.1</v>
       </c>
       <c r="D12" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E12" t="n">
         <v>0.7</v>
       </c>
       <c r="F12" t="n">
-        <v>36.37736208925489</v>
+        <v>28.468194206537667</v>
       </c>
       <c r="G12" t="n">
-        <v>19.72082422164684</v>
+        <v>15.321681351307507</v>
       </c>
       <c r="H12" t="n">
-        <v>12.542446832545481</v>
+        <v>10.475406341939857</v>
       </c>
       <c r="I12" t="n">
-        <v>234.28174360141236</v>
+        <v>195.27643044466652</v>
       </c>
       <c r="J12" t="n">
-        <v>189.40744060235656</v>
+        <v>148.4084138254848</v>
       </c>
       <c r="K12" t="n">
-        <v>111.67769253169617</v>
+        <v>106.07114746163245</v>
       </c>
       <c r="L12" t="n">
         <v>0.0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.9976882447156205</v>
+        <v>0.9486289471915826</v>
       </c>
       <c r="N12" t="n">
-        <v>1.1536033054933545</v>
+        <v>0.9615411435095379</v>
       </c>
       <c r="O12" t="n">
-        <v>0.9326422375260046</v>
+        <v>0.7307630296766873</v>
       </c>
       <c r="P12" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5222943301010782</v>
       </c>
       <c r="Q12" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R12" t="n">
-        <v>1.125E7</v>
+        <v>900000.0</v>
       </c>
       <c r="S12" t="n">
         <v>0.08</v>
@@ -896,49 +896,49 @@
         <v>0.1</v>
       </c>
       <c r="D13" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E13" t="n">
         <v>0.7</v>
       </c>
       <c r="F13" t="n">
-        <v>36.32724754227387</v>
+        <v>29.13416263451292</v>
       </c>
       <c r="G13" t="n">
-        <v>19.719062606681838</v>
+        <v>15.526753750239736</v>
       </c>
       <c r="H13" t="n">
-        <v>12.543517691994522</v>
+        <v>10.493498865737985</v>
       </c>
       <c r="I13" t="n">
-        <v>234.2758412568632</v>
+        <v>195.27840153292237</v>
       </c>
       <c r="J13" t="n">
-        <v>189.39552690947448</v>
+        <v>148.30192685288173</v>
       </c>
       <c r="K13" t="n">
-        <v>111.67769253169617</v>
+        <v>105.98649796640085</v>
       </c>
       <c r="L13" t="n">
         <v>0.0</v>
       </c>
       <c r="M13" t="n">
-        <v>0.9975675674123955</v>
+        <v>0.9486734775409391</v>
       </c>
       <c r="N13" t="n">
-        <v>1.1535742423487945</v>
+        <v>0.9615508491481097</v>
       </c>
       <c r="O13" t="n">
-        <v>0.9325835745022533</v>
+        <v>0.7302386878235895</v>
       </c>
       <c r="P13" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5218775159865577</v>
       </c>
       <c r="Q13" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R13" t="n">
-        <v>7650000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="S13" t="n">
         <v>0.08</v>
@@ -961,49 +961,49 @@
         <v>0.1</v>
       </c>
       <c r="D14" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E14" t="n">
         <v>0.7</v>
       </c>
       <c r="F14" t="n">
-        <v>36.36486944915575</v>
+        <v>28.449483016285107</v>
       </c>
       <c r="G14" t="n">
-        <v>19.720530313127536</v>
+        <v>15.392288194838935</v>
       </c>
       <c r="H14" t="n">
-        <v>12.542730194845157</v>
+        <v>10.483263075215659</v>
       </c>
       <c r="I14" t="n">
-        <v>234.28025208397867</v>
+        <v>195.27736993495424</v>
       </c>
       <c r="J14" t="n">
-        <v>189.40400524188064</v>
+        <v>148.35418052169572</v>
       </c>
       <c r="K14" t="n">
-        <v>111.67769253169617</v>
+        <v>106.02882271401666</v>
       </c>
       <c r="L14" t="n">
         <v>0.0</v>
       </c>
       <c r="M14" t="n">
-        <v>0.9976577496640167</v>
+        <v>0.9486501719290366</v>
       </c>
       <c r="N14" t="n">
-        <v>1.153595961261511</v>
+        <v>0.9615457695597147</v>
       </c>
       <c r="O14" t="n">
-        <v>0.9326253218110199</v>
+        <v>0.7304959848888299</v>
       </c>
       <c r="P14" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5220859230438181</v>
       </c>
       <c r="Q14" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R14" t="n">
-        <v>1.035E7</v>
+        <v>900000.0</v>
       </c>
       <c r="S14" t="n">
         <v>0.08</v>
@@ -1026,49 +1026,49 @@
         <v>0.1</v>
       </c>
       <c r="D15" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E15" t="n">
         <v>0.7</v>
       </c>
       <c r="F15" t="n">
-        <v>36.389830948775696</v>
+        <v>28.4774638166753</v>
       </c>
       <c r="G15" t="n">
-        <v>19.72112871562885</v>
+        <v>15.294953590407099</v>
       </c>
       <c r="H15" t="n">
-        <v>12.542161354172922</v>
+        <v>10.478897420579605</v>
       </c>
       <c r="I15" t="n">
-        <v>234.28324573971037</v>
+        <v>195.28397982583473</v>
       </c>
       <c r="J15" t="n">
-        <v>189.41088307839755</v>
+        <v>148.4347679942225</v>
       </c>
       <c r="K15" t="n">
-        <v>111.67769253169617</v>
+        <v>106.09230983544036</v>
       </c>
       <c r="L15" t="n">
         <v>0.0</v>
       </c>
       <c r="M15" t="n">
-        <v>0.997718956917756</v>
+        <v>0.9487995009858382</v>
       </c>
       <c r="N15" t="n">
-        <v>1.1536107020223338</v>
+        <v>0.9615783166624102</v>
       </c>
       <c r="O15" t="n">
-        <v>0.9326591882780289</v>
+        <v>0.7308927976035517</v>
       </c>
       <c r="P15" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5223985336297083</v>
       </c>
       <c r="Q15" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R15" t="n">
-        <v>1.215E7</v>
+        <v>900000.0</v>
       </c>
       <c r="S15" t="n">
         <v>0.08</v>
@@ -1091,49 +1091,49 @@
         <v>0.1</v>
       </c>
       <c r="D16" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E16" t="n">
         <v>0.7</v>
       </c>
       <c r="F16" t="n">
-        <v>36.40227615661695</v>
+        <v>28.775298075243033</v>
       </c>
       <c r="G16" t="n">
-        <v>19.722055968276596</v>
+        <v>15.24550006088727</v>
       </c>
       <c r="H16" t="n">
-        <v>12.541854323807447</v>
+        <v>10.471664524462325</v>
       </c>
       <c r="I16" t="n">
-        <v>234.28475849887255</v>
+        <v>195.2813985221127</v>
       </c>
       <c r="J16" t="n">
-        <v>189.41265058338158</v>
+        <v>148.48313559314437</v>
       </c>
       <c r="K16" t="n">
-        <v>111.67769253169617</v>
+        <v>106.11347220924827</v>
       </c>
       <c r="L16" t="n">
         <v>0.0</v>
       </c>
       <c r="M16" t="n">
-        <v>0.9977498862704234</v>
+        <v>0.9487411847961925</v>
       </c>
       <c r="N16" t="n">
-        <v>1.1536181508484484</v>
+        <v>0.961565606322883</v>
       </c>
       <c r="O16" t="n">
-        <v>0.9326678914725718</v>
+        <v>0.7311309596606431</v>
       </c>
       <c r="P16" t="n">
-        <v>0.549900958026072</v>
+        <v>0.5225027371583385</v>
       </c>
       <c r="Q16" t="n">
-        <v>25.0</v>
+        <v>35.0</v>
       </c>
       <c r="R16" t="n">
-        <v>1.305E7</v>
+        <v>900000.0</v>
       </c>
       <c r="S16" t="n">
         <v>0.08</v>
@@ -1142,71 +1142,6 @@
         <v>39.39</v>
       </c>
       <c r="U16" t="n">
-        <v>1458.0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>30.0</v>
-      </c>
-      <c r="B17" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F17" t="n">
-        <v>36.414697840747564</v>
-      </c>
-      <c r="G17" t="n">
-        <v>19.72238124211358</v>
-      </c>
-      <c r="H17" t="n">
-        <v>12.541564615497116</v>
-      </c>
-      <c r="I17" t="n">
-        <v>234.28628187889905</v>
-      </c>
-      <c r="J17" t="n">
-        <v>189.41610729055174</v>
-      </c>
-      <c r="K17" t="n">
-        <v>111.67769253169617</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.9977810327736225</v>
-      </c>
-      <c r="N17" t="n">
-        <v>1.153625651971699</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0.932684912298677</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0.549900958026072</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>25.0</v>
-      </c>
-      <c r="R17" t="n">
-        <v>1.395E7</v>
-      </c>
-      <c r="S17" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="T17" t="n">
-        <v>39.39</v>
-      </c>
-      <c r="U17" t="n">
         <v>1458.0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Starting capacity experiment executed. Results in Book1.
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -60,7 +60,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -169,6 +169,11 @@
           <t>fixed opex</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>starting capacity</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -187,37 +192,37 @@
         <v>0.7</v>
       </c>
       <c r="F2" t="n">
-        <v>28.41097645332293</v>
+        <v>29.473923819084238</v>
       </c>
       <c r="G2" t="n">
-        <v>16.50237684348026</v>
+        <v>16.63690746801699</v>
       </c>
       <c r="H2" t="n">
-        <v>10.545823234677838</v>
+        <v>10.552466485108072</v>
       </c>
       <c r="I2" t="n">
-        <v>195.2795744295943</v>
+        <v>195.27244450605397</v>
       </c>
       <c r="J2" t="n">
-        <v>147.5371247524124</v>
+        <v>147.44248471645096</v>
       </c>
       <c r="K2" t="n">
-        <v>105.94417321878504</v>
+        <v>105.92301084497716</v>
       </c>
       <c r="L2" t="n">
         <v>0.0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9486999753389981</v>
+        <v>0.9485388978300666</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9615566244913223</v>
+        <v>0.9615215167478097</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7264728022808785</v>
+        <v>0.7260067947438049</v>
       </c>
       <c r="P2" t="n">
-        <v>0.5216691089292975</v>
+        <v>0.5215649054006675</v>
       </c>
       <c r="Q2" t="n">
         <v>35.0</v>
@@ -233,6 +238,9 @@
       </c>
       <c r="U2" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>55000.0</v>
       </c>
     </row>
     <row r="3">
@@ -252,37 +260,37 @@
         <v>0.7</v>
       </c>
       <c r="F3" t="n">
-        <v>29.780783977693822</v>
+        <v>28.41097645332293</v>
       </c>
       <c r="G3" t="n">
-        <v>15.58365163678584</v>
+        <v>16.50237684348026</v>
       </c>
       <c r="H3" t="n">
-        <v>10.496061526398798</v>
+        <v>10.545823234677838</v>
       </c>
       <c r="I3" t="n">
-        <v>195.28693645821852</v>
+        <v>195.2795744295943</v>
       </c>
       <c r="J3" t="n">
-        <v>148.27430970996303</v>
+        <v>147.5371247524124</v>
       </c>
       <c r="K3" t="n">
-        <v>105.96533559259294</v>
+        <v>105.94417321878504</v>
       </c>
       <c r="L3" t="n">
         <v>0.0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9488662965098728</v>
+        <v>0.9486999753389981</v>
       </c>
       <c r="N3" t="n">
-        <v>0.9615928751202679</v>
+        <v>0.9615566244913223</v>
       </c>
       <c r="O3" t="n">
-        <v>0.730102701011858</v>
+        <v>0.7264728022808785</v>
       </c>
       <c r="P3" t="n">
-        <v>0.5217733124579276</v>
+        <v>0.5216691089292975</v>
       </c>
       <c r="Q3" t="n">
         <v>35.0</v>
@@ -298,6 +306,9 @@
       </c>
       <c r="U3" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>60000.0</v>
       </c>
     </row>
     <row r="4">
@@ -317,37 +328,37 @@
         <v>0.7</v>
       </c>
       <c r="F4" t="n">
-        <v>29.969710495299793</v>
+        <v>29.780783977693822</v>
       </c>
       <c r="G4" t="n">
-        <v>16.964644979867217</v>
+        <v>15.58365163678584</v>
       </c>
       <c r="H4" t="n">
-        <v>10.60809208186763</v>
+        <v>10.496061526398798</v>
       </c>
       <c r="I4" t="n">
-        <v>195.2790628606574</v>
+        <v>195.28693645821852</v>
       </c>
       <c r="J4" t="n">
-        <v>146.95659545461845</v>
+        <v>148.27430970996303</v>
       </c>
       <c r="K4" t="n">
-        <v>105.81719897593761</v>
+        <v>105.96533559259294</v>
       </c>
       <c r="L4" t="n">
         <v>0.0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9486884180972501</v>
+        <v>0.9488662965098728</v>
       </c>
       <c r="N4" t="n">
-        <v>0.9615541055258771</v>
+        <v>0.9615928751202679</v>
       </c>
       <c r="O4" t="n">
-        <v>0.7236142760185416</v>
+        <v>0.730102701011858</v>
       </c>
       <c r="P4" t="n">
-        <v>0.5210438877575169</v>
+        <v>0.5217733124579276</v>
       </c>
       <c r="Q4" t="n">
         <v>35.0</v>
@@ -363,6 +374,9 @@
       </c>
       <c r="U4" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>65000.0</v>
       </c>
     </row>
     <row r="5">
@@ -382,37 +396,37 @@
         <v>0.7</v>
       </c>
       <c r="F5" t="n">
-        <v>30.21357635776602</v>
+        <v>29.969710495299793</v>
       </c>
       <c r="G5" t="n">
-        <v>16.694586352223947</v>
+        <v>16.964644979867217</v>
       </c>
       <c r="H5" t="n">
-        <v>10.553937002892145</v>
+        <v>10.60809208186763</v>
       </c>
       <c r="I5" t="n">
-        <v>195.28145804737852</v>
+        <v>195.2790628606574</v>
       </c>
       <c r="J5" t="n">
-        <v>147.3502025453923</v>
+        <v>146.95659545461845</v>
       </c>
       <c r="K5" t="n">
-        <v>105.90184847116923</v>
+        <v>105.81719897593761</v>
       </c>
       <c r="L5" t="n">
         <v>0.0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.9487425295766067</v>
+        <v>0.9486884180972501</v>
       </c>
       <c r="N5" t="n">
-        <v>0.9615658994252918</v>
+        <v>0.9615541055258771</v>
       </c>
       <c r="O5" t="n">
-        <v>0.7255523973335115</v>
+        <v>0.7236142760185416</v>
       </c>
       <c r="P5" t="n">
-        <v>0.5214607018720373</v>
+        <v>0.5210438877575169</v>
       </c>
       <c r="Q5" t="n">
         <v>35.0</v>
@@ -428,6 +442,9 @@
       </c>
       <c r="U5" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>30000.0</v>
       </c>
     </row>
     <row r="6">
@@ -447,37 +464,37 @@
         <v>0.7</v>
       </c>
       <c r="F6" t="n">
-        <v>29.473923819084238</v>
+        <v>30.21357635776602</v>
       </c>
       <c r="G6" t="n">
-        <v>16.63690746801699</v>
+        <v>16.694586352223947</v>
       </c>
       <c r="H6" t="n">
-        <v>10.552466485108072</v>
+        <v>10.553937002892145</v>
       </c>
       <c r="I6" t="n">
-        <v>195.27244450605397</v>
+        <v>195.28145804737852</v>
       </c>
       <c r="J6" t="n">
-        <v>147.44248471645096</v>
+        <v>147.3502025453923</v>
       </c>
       <c r="K6" t="n">
-        <v>105.92301084497716</v>
+        <v>105.90184847116923</v>
       </c>
       <c r="L6" t="n">
         <v>0.0</v>
       </c>
       <c r="M6" t="n">
-        <v>0.9485388978300666</v>
+        <v>0.9487425295766067</v>
       </c>
       <c r="N6" t="n">
-        <v>0.9615215167478097</v>
+        <v>0.9615658994252918</v>
       </c>
       <c r="O6" t="n">
-        <v>0.7260067947438049</v>
+        <v>0.7255523973335115</v>
       </c>
       <c r="P6" t="n">
-        <v>0.5215649054006675</v>
+        <v>0.5214607018720373</v>
       </c>
       <c r="Q6" t="n">
         <v>35.0</v>
@@ -493,6 +510,9 @@
       </c>
       <c r="U6" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>50000.0</v>
       </c>
     </row>
     <row r="7">
@@ -559,6 +579,9 @@
       <c r="U7" t="n">
         <v>1458.0</v>
       </c>
+      <c r="V7" t="n">
+        <v>45000.0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -624,6 +647,9 @@
       <c r="U8" t="n">
         <v>1458.0</v>
       </c>
+      <c r="V8" t="n">
+        <v>40000.0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -642,37 +668,37 @@
         <v>0.7</v>
       </c>
       <c r="F9" t="n">
-        <v>28.56673852253458</v>
+        <v>29.867460380569</v>
       </c>
       <c r="G9" t="n">
-        <v>15.478079803252363</v>
+        <v>16.880881194352394</v>
       </c>
       <c r="H9" t="n">
-        <v>10.496878473593608</v>
+        <v>10.605308784976822</v>
       </c>
       <c r="I9" t="n">
-        <v>195.28585880641012</v>
+        <v>195.27341471283276</v>
       </c>
       <c r="J9" t="n">
-        <v>148.32820990917693</v>
+        <v>147.04566799527734</v>
       </c>
       <c r="K9" t="n">
-        <v>106.00766034020876</v>
+        <v>105.83836134974551</v>
       </c>
       <c r="L9" t="n">
         <v>0.0</v>
       </c>
       <c r="M9" t="n">
-        <v>0.9488419504607455</v>
+        <v>0.9485608165070605</v>
       </c>
       <c r="N9" t="n">
-        <v>0.9615875687627634</v>
+        <v>0.9615262940459884</v>
       </c>
       <c r="O9" t="n">
-        <v>0.7303681055927874</v>
+        <v>0.7240528692087459</v>
       </c>
       <c r="P9" t="n">
-        <v>0.521981719515188</v>
+        <v>0.5211480912861469</v>
       </c>
       <c r="Q9" t="n">
         <v>35.0</v>
@@ -688,6 +714,9 @@
       </c>
       <c r="U9" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>35000.0</v>
       </c>
     </row>
     <row r="10">
@@ -707,37 +736,37 @@
         <v>0.7</v>
       </c>
       <c r="F10" t="n">
-        <v>29.867460380569</v>
+        <v>28.56673852253458</v>
       </c>
       <c r="G10" t="n">
-        <v>16.880881194352394</v>
+        <v>15.478079803252363</v>
       </c>
       <c r="H10" t="n">
-        <v>10.605308784976822</v>
+        <v>10.496878473593608</v>
       </c>
       <c r="I10" t="n">
-        <v>195.27341471283276</v>
+        <v>195.28585880641012</v>
       </c>
       <c r="J10" t="n">
-        <v>147.04566799527734</v>
+        <v>148.32820990917693</v>
       </c>
       <c r="K10" t="n">
-        <v>105.83836134974551</v>
+        <v>106.00766034020876</v>
       </c>
       <c r="L10" t="n">
         <v>0.0</v>
       </c>
       <c r="M10" t="n">
-        <v>0.9485608165070605</v>
+        <v>0.9488419504607455</v>
       </c>
       <c r="N10" t="n">
-        <v>0.9615262940459884</v>
+        <v>0.9615875687627634</v>
       </c>
       <c r="O10" t="n">
-        <v>0.7240528692087459</v>
+        <v>0.7303681055927874</v>
       </c>
       <c r="P10" t="n">
-        <v>0.5211480912861469</v>
+        <v>0.521981719515188</v>
       </c>
       <c r="Q10" t="n">
         <v>35.0</v>
@@ -753,6 +782,9 @@
       </c>
       <c r="U10" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V10" t="n">
+        <v>75000.0</v>
       </c>
     </row>
     <row r="11">
@@ -772,37 +804,37 @@
         <v>0.7</v>
       </c>
       <c r="F11" t="n">
-        <v>28.45887060621136</v>
+        <v>29.13416263451292</v>
       </c>
       <c r="G11" t="n">
-        <v>15.351650585600195</v>
+        <v>15.526753750239736</v>
       </c>
       <c r="H11" t="n">
-        <v>10.47846629169804</v>
+        <v>10.493498865737985</v>
       </c>
       <c r="I11" t="n">
-        <v>195.28487326228222</v>
+        <v>195.27840153292237</v>
       </c>
       <c r="J11" t="n">
-        <v>148.3824076567449</v>
+        <v>148.30192685288173</v>
       </c>
       <c r="K11" t="n">
-        <v>106.04998508782455</v>
+        <v>105.98649796640085</v>
       </c>
       <c r="L11" t="n">
         <v>0.0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.9488196852860675</v>
+        <v>0.9486734775409391</v>
       </c>
       <c r="N11" t="n">
-        <v>0.9615827159434777</v>
+        <v>0.9615508491481097</v>
       </c>
       <c r="O11" t="n">
-        <v>0.7306349753018117</v>
+        <v>0.7302386878235895</v>
       </c>
       <c r="P11" t="n">
-        <v>0.5221901265724481</v>
+        <v>0.5218775159865577</v>
       </c>
       <c r="Q11" t="n">
         <v>35.0</v>
@@ -818,6 +850,9 @@
       </c>
       <c r="U11" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V11" t="n">
+        <v>70000.0</v>
       </c>
     </row>
     <row r="12">
@@ -837,37 +872,37 @@
         <v>0.7</v>
       </c>
       <c r="F12" t="n">
-        <v>28.468194206537667</v>
+        <v>28.449483016285107</v>
       </c>
       <c r="G12" t="n">
-        <v>15.321681351307507</v>
+        <v>15.392288194838935</v>
       </c>
       <c r="H12" t="n">
-        <v>10.475406341939857</v>
+        <v>10.483263075215659</v>
       </c>
       <c r="I12" t="n">
-        <v>195.27643044466652</v>
+        <v>195.27736993495424</v>
       </c>
       <c r="J12" t="n">
-        <v>148.4084138254848</v>
+        <v>148.35418052169572</v>
       </c>
       <c r="K12" t="n">
-        <v>106.07114746163245</v>
+        <v>106.02882271401666</v>
       </c>
       <c r="L12" t="n">
         <v>0.0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.9486289471915826</v>
+        <v>0.9486501719290366</v>
       </c>
       <c r="N12" t="n">
-        <v>0.9615411435095379</v>
+        <v>0.9615457695597147</v>
       </c>
       <c r="O12" t="n">
-        <v>0.7307630296766873</v>
+        <v>0.7304959848888299</v>
       </c>
       <c r="P12" t="n">
-        <v>0.5222943301010782</v>
+        <v>0.5220859230438181</v>
       </c>
       <c r="Q12" t="n">
         <v>35.0</v>
@@ -883,6 +918,9 @@
       </c>
       <c r="U12" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V12" t="n">
+        <v>80000.0</v>
       </c>
     </row>
     <row r="13">
@@ -902,37 +940,37 @@
         <v>0.7</v>
       </c>
       <c r="F13" t="n">
-        <v>29.13416263451292</v>
+        <v>28.45887060621136</v>
       </c>
       <c r="G13" t="n">
-        <v>15.526753750239736</v>
+        <v>15.351650585600195</v>
       </c>
       <c r="H13" t="n">
-        <v>10.493498865737985</v>
+        <v>10.47846629169804</v>
       </c>
       <c r="I13" t="n">
-        <v>195.27840153292237</v>
+        <v>195.28487326228222</v>
       </c>
       <c r="J13" t="n">
-        <v>148.30192685288173</v>
+        <v>148.3824076567449</v>
       </c>
       <c r="K13" t="n">
-        <v>105.98649796640085</v>
+        <v>106.04998508782455</v>
       </c>
       <c r="L13" t="n">
         <v>0.0</v>
       </c>
       <c r="M13" t="n">
-        <v>0.9486734775409391</v>
+        <v>0.9488196852860675</v>
       </c>
       <c r="N13" t="n">
-        <v>0.9615508491481097</v>
+        <v>0.9615827159434777</v>
       </c>
       <c r="O13" t="n">
-        <v>0.7302386878235895</v>
+        <v>0.7306349753018117</v>
       </c>
       <c r="P13" t="n">
-        <v>0.5218775159865577</v>
+        <v>0.5221901265724481</v>
       </c>
       <c r="Q13" t="n">
         <v>35.0</v>
@@ -948,6 +986,9 @@
       </c>
       <c r="U13" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V13" t="n">
+        <v>85000.0</v>
       </c>
     </row>
     <row r="14">
@@ -967,37 +1008,37 @@
         <v>0.7</v>
       </c>
       <c r="F14" t="n">
-        <v>28.449483016285107</v>
+        <v>28.468194206537667</v>
       </c>
       <c r="G14" t="n">
-        <v>15.392288194838935</v>
+        <v>15.321681351307507</v>
       </c>
       <c r="H14" t="n">
-        <v>10.483263075215659</v>
+        <v>10.475406341939857</v>
       </c>
       <c r="I14" t="n">
-        <v>195.27736993495424</v>
+        <v>195.27643044466652</v>
       </c>
       <c r="J14" t="n">
-        <v>148.35418052169572</v>
+        <v>148.4084138254848</v>
       </c>
       <c r="K14" t="n">
-        <v>106.02882271401666</v>
+        <v>106.07114746163245</v>
       </c>
       <c r="L14" t="n">
         <v>0.0</v>
       </c>
       <c r="M14" t="n">
-        <v>0.9486501719290366</v>
+        <v>0.9486289471915826</v>
       </c>
       <c r="N14" t="n">
-        <v>0.9615457695597147</v>
+        <v>0.9615411435095379</v>
       </c>
       <c r="O14" t="n">
-        <v>0.7304959848888299</v>
+        <v>0.7307630296766873</v>
       </c>
       <c r="P14" t="n">
-        <v>0.5220859230438181</v>
+        <v>0.5222943301010782</v>
       </c>
       <c r="Q14" t="n">
         <v>35.0</v>
@@ -1013,6 +1054,9 @@
       </c>
       <c r="U14" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V14" t="n">
+        <v>90000.0</v>
       </c>
     </row>
     <row r="15">
@@ -1079,6 +1123,9 @@
       <c r="U15" t="n">
         <v>1458.0</v>
       </c>
+      <c r="V15" t="n">
+        <v>95000.0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1143,6 +1190,9 @@
       </c>
       <c r="U16" t="n">
         <v>1458.0</v>
+      </c>
+      <c r="V16" t="n">
+        <v>100000.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>